<commit_message>
Add iLogic extractors and CAD updates
- cad/ilogic/extract_model.iLogicVb, extract_pose_and_solve.iLogicVb
- cad/drawings/knee_shaft.pdf
- cad/reports/static momentum/{4,6}point.iaa
- cad/leg_tibea/shaft_tibea.idw
- updated body/leg parts and FEA artifacts

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cad/parametres.xlsx
+++ b/cad/parametres.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\spider_metal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{001E5629-F010-42F5-B47E-ABC710F5AE44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8CDA13E-B1AC-4169-9E43-7A178E8DB6BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1500" yWindow="1500" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="45">
   <si>
     <t>d_main_shaft</t>
   </si>
@@ -160,6 +160,9 @@
   </si>
   <si>
     <t>hight_ground_clearance</t>
+  </si>
+  <si>
+    <t>16mm</t>
   </si>
 </sst>
 </file>
@@ -512,7 +515,7 @@
         <v>0</v>
       </c>
       <c r="B4" t="s">
-        <v>3</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Update CAD: new leg parts, screws, FEA on right tibea
- New parts: tibea_thorn_profile, tibea_reinforcement(2)_steel,
  tibea_ring_for_bearing_tibea, femur_reinforcement_tibea_steel,
  bearing_unit_15mm
- Removed tibea_inside_steel
- Added cad/screw/ (M6 bolts/nut)
- Added FEA results for leg_Right_tibea_ass/
- Updated body, leg assemblies and existing parts

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cad/parametres.xlsx
+++ b/cad/parametres.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\spider_metal\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\vs_code_projects\ogonek-spider\physical-structure\cad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8CDA13E-B1AC-4169-9E43-7A178E8DB6BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AFEC5A2-84D4-4CA1-9AE2-3B72DC1B9C00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -75,9 +75,6 @@
     <t>thickness_steel</t>
   </si>
   <si>
-    <t>4mm</t>
-  </si>
-  <si>
     <t>width_profile_femur</t>
   </si>
   <si>
@@ -162,7 +159,10 @@
     <t>hight_ground_clearance</t>
   </si>
   <si>
-    <t>16mm</t>
+    <t>15mm</t>
+  </si>
+  <si>
+    <t>37mm</t>
   </si>
 </sst>
 </file>
@@ -507,7 +507,7 @@
         <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
@@ -515,15 +515,15 @@
         <v>0</v>
       </c>
       <c r="B4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
@@ -531,7 +531,7 @@
         <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
@@ -568,23 +568,23 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" t="s">
         <v>16</v>
-      </c>
-      <c r="B11" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B12" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B13" t="s">
         <v>12</v>
@@ -592,47 +592,47 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B14" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15" t="s">
         <v>21</v>
-      </c>
-      <c r="B15" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B16" t="s">
-        <v>2</v>
+        <v>44</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B17" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B18" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B19" t="s">
         <v>2</v>
@@ -640,50 +640,50 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
+        <v>31</v>
+      </c>
+      <c r="B20" t="s">
         <v>32</v>
-      </c>
-      <c r="B20" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B21" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B22" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B23" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B24" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B25" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rework knee joint for 20mm shaft
- Replaced bearing_unit_15mm with bearing_unit_20mm
- Updated femur/tibea parts and assemblies for the new shaft size
- Added DXF drawings under cad/drawings/knee_joint and knee_joint_20mm
- Refreshed FEA results for leg_Right_tibea_ass

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cad/parametres.xlsx
+++ b/cad/parametres.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\vs_code_projects\ogonek-spider\physical-structure\cad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AFEC5A2-84D4-4CA1-9AE2-3B72DC1B9C00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45C74C51-4D9C-4148-9529-2D672654B4FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1500" yWindow="1500" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="44">
   <si>
     <t>d_main_shaft</t>
   </si>
@@ -157,9 +157,6 @@
   </si>
   <si>
     <t>hight_ground_clearance</t>
-  </si>
-  <si>
-    <t>15mm</t>
   </si>
   <si>
     <t>37mm</t>
@@ -515,7 +512,7 @@
         <v>0</v>
       </c>
       <c r="B4" t="s">
-        <v>43</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
@@ -611,7 +608,7 @@
         <v>22</v>
       </c>
       <c r="B16" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">

</xml_diff>